<commit_message>
replace DHW data; fix bioerosion readme typo
</commit_message>
<xml_diff>
--- a/www/Bioerosion_Data_EXAMPLE.xlsx
+++ b/www/Bioerosion_Data_EXAMPLE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0770CA7E-5685-4C6A-BFC1-42D29D7B042A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{173BFBD2-5B8D-4D68-8744-1BCCC791019D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="14566" windowHeight="7822" activeTab="1" xr2:uid="{19050643-5FB9-4299-B24C-C8F9EBB4329D}"/>
+    <workbookView xWindow="0" yWindow="2205" windowWidth="28905" windowHeight="11190" xr2:uid="{19050643-5FB9-4299-B24C-C8F9EBB4329D}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
@@ -163,9 +163,6 @@
     <t xml:space="preserve">•  Sponges abundance should be quantified as total area in centimeters squared (cm2) occupied by each species; if survey data is instead in percent cover, it should be converted to area by multiplying the percent cover by Survey_Area_Sponges_m2 and then multiplying by 10,000 to covert m2 to cm2 </t>
   </si>
   <si>
-    <t xml:space="preserve">• Provide the area (in meters squared [m2]) where urchin surveys were conducted in Survey_Area_Sponges_m2; For example a 1 x 10 m belt transect would have a 10 m2 survey area </t>
-  </si>
-  <si>
     <t>Survey_Area_Sponges_m2</t>
   </si>
   <si>
@@ -248,6 +245,9 @@
   </si>
   <si>
     <t>Cliona delitrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Provide the area (in meters squared [m2]) where sponge surveys were conducted in Survey_Area_Sponges_m2; For example a 1 x 10 m belt transect would have a 10 m2 survey area </t>
   </si>
 </sst>
 </file>
@@ -758,7 +758,7 @@
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -799,21 +799,21 @@
         <v>21</v>
       </c>
       <c r="G1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" t="s">
         <v>30</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" t="s">
-        <v>31</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -827,16 +827,16 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" t="s">
         <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" t="s">
-        <v>31</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -850,16 +850,16 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -873,16 +873,16 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" t="s">
         <v>32</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -896,16 +896,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -919,16 +919,16 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" t="s">
         <v>37</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" t="s">
-        <v>38</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -942,16 +942,16 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -965,16 +965,16 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -988,16 +988,16 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" t="s">
         <v>30</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" t="s">
-        <v>31</v>
       </c>
       <c r="E10">
         <v>4</v>
@@ -1011,16 +1011,16 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -1034,16 +1034,16 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" t="s">
         <v>32</v>
-      </c>
-      <c r="D12" t="s">
-        <v>33</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -1057,16 +1057,16 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" t="s">
         <v>32</v>
-      </c>
-      <c r="D13" t="s">
-        <v>33</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -1080,16 +1080,16 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -1103,16 +1103,16 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -1126,16 +1126,16 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -1149,16 +1149,16 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E17">
         <v>2</v>
@@ -1172,16 +1172,16 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" t="s">
         <v>32</v>
-      </c>
-      <c r="D18" t="s">
-        <v>33</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -1195,16 +1195,16 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" t="s">
         <v>37</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" t="s">
-        <v>38</v>
       </c>
       <c r="E19">
         <v>2</v>
@@ -1218,16 +1218,16 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C20" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" t="s">
         <v>32</v>
-      </c>
-      <c r="D20" t="s">
-        <v>33</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -1241,16 +1241,16 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" t="s">
         <v>32</v>
-      </c>
-      <c r="D21" t="s">
-        <v>33</v>
       </c>
       <c r="E21">
         <v>2</v>
@@ -1264,16 +1264,16 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C22" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" t="s">
         <v>32</v>
-      </c>
-      <c r="D22" t="s">
-        <v>33</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -1287,16 +1287,16 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" t="s">
         <v>30</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D23" t="s">
-        <v>31</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -1310,16 +1310,16 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B24" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E24">
         <v>4</v>
@@ -1333,16 +1333,16 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -1356,16 +1356,16 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C26" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D26" t="s">
         <v>32</v>
-      </c>
-      <c r="D26" t="s">
-        <v>33</v>
       </c>
       <c r="E26">
         <v>4</v>
@@ -1379,16 +1379,16 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -1402,16 +1402,16 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" t="s">
         <v>32</v>
-      </c>
-      <c r="D28" t="s">
-        <v>33</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -1425,16 +1425,16 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B29" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -1448,16 +1448,16 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -1471,16 +1471,16 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -1494,16 +1494,16 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B32" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -1517,16 +1517,16 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E33">
         <v>3</v>
@@ -1540,16 +1540,16 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B34" t="s">
+        <v>36</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D34" t="s">
         <v>37</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D34" t="s">
-        <v>38</v>
       </c>
       <c r="E34">
         <v>2</v>
@@ -1563,16 +1563,16 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E35">
         <v>1</v>
@@ -1586,16 +1586,16 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E36">
         <v>1</v>
@@ -1654,18 +1654,18 @@
         <v>22</v>
       </c>
       <c r="F1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" t="s">
         <v>51</v>
-      </c>
-      <c r="C2" t="s">
-        <v>52</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1679,13 +1679,13 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" t="s">
         <v>53</v>
-      </c>
-      <c r="C3" t="s">
-        <v>54</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -1699,13 +1699,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
         <v>53</v>
-      </c>
-      <c r="C4" t="s">
-        <v>54</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1719,13 +1719,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1739,13 +1739,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s">
         <v>53</v>
-      </c>
-      <c r="C6" t="s">
-        <v>54</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -1792,18 +1792,18 @@
         <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C2">
         <v>50</v>
@@ -1817,10 +1817,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C3">
         <v>5</v>
@@ -1834,10 +1834,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -1851,10 +1851,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -1868,10 +1868,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C6">
         <v>7</v>
@@ -1885,10 +1885,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C7">
         <v>4</v>
@@ -1902,10 +1902,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C8">
         <v>5</v>
@@ -1919,10 +1919,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9">
         <v>4</v>
@@ -1936,10 +1936,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -1953,10 +1953,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -1970,10 +1970,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C12">
         <v>6</v>
@@ -2005,6 +2005,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="647735499ae6baa62e6fc7f5ed3567b4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="47ff4a2bf1fedf465812d90a21a07c12" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
@@ -2199,17 +2210,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A206479D-07AC-477F-8545-4966E63B8E30}">
   <ds:schemaRefs>
@@ -2219,6 +2219,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FB6342C-EC7C-49F8-97E7-6339AB75B937}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
+    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02949C9A-F615-4134-92DC-033BFA8951F4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2237,17 +2248,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FB6342C-EC7C-49F8-97E7-6339AB75B937}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
-    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>

</xml_diff>